<commit_message>
remove the unused jeepney files and the old pagasa client
the engine builds the jeepney layer from virtual_stops.geojson, so
split_jeepneys.py, the two discretized json files and
jeepney_stops_no_300m.geojson were never read. deleted them and the
middle graph tier that loaded them. SCPH_GEOJSON=0 now goes straight to
the coarse 10-anchor graph.

the panel approved met norway as the rainfall source, so the dormant
pagasa client, its token variable and its parser are gone, and
fetch_pagasa_rainfall_mm is now fetch_rainfall_mm. the safest profile card
and the researcher dashboard chip name met norway. docs/rainfall-source.md
replaces the old request note.

routing output is unchanged: every api output was hashed before and after
(180 routes, 45 compares, network, benchmark) and the hashes match.
</commit_message>
<xml_diff>
--- a/Group11_Delegation_Timeline.xlsx
+++ b/Group11_Delegation_Timeline.xlsx
@@ -23,9 +23,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="ddd mmm d"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="ddd mmm d"/>
   </numFmts>
   <fonts count="18">
     <font>
@@ -190,7 +189,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -212,11 +211,55 @@
         <color rgb="00D9DEE7"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D9DEE7"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D9DEE7"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9DEE7"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D9DEE7"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9DEE7"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D9DEE7"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9DEE7"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9DEE7"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -299,7 +342,7 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -320,7 +363,7 @@
     <xf numFmtId="0" fontId="15" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="4" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -352,6 +395,14 @@
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -752,6 +803,8 @@
           <t>Working prototype for panel — finished the soonest (target ~1 month: Jul 13 - Aug 15).</t>
         </is>
       </c>
+      <c r="C4" s="46" t="n"/>
+      <c r="D4" s="47" t="n"/>
     </row>
     <row r="5" ht="26" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
@@ -764,6 +817,8 @@
           <t>Monday, July 13, 2026 (kickoff meeting)</t>
         </is>
       </c>
+      <c r="C5" s="46" t="n"/>
+      <c r="D5" s="47" t="n"/>
     </row>
     <row r="6" ht="26" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
@@ -776,6 +831,8 @@
           <t>Every Saturday — Jul 18, Jul 25, Aug 1, Aug 8, Aug 15</t>
         </is>
       </c>
+      <c r="C6" s="46" t="n"/>
+      <c r="D6" s="47" t="n"/>
     </row>
     <row r="7" ht="26" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
@@ -788,6 +845,8 @@
           <t>Saturday, July 18, 2026 (hard sub-deadline)</t>
         </is>
       </c>
+      <c r="C7" s="46" t="n"/>
+      <c r="D7" s="47" t="n"/>
     </row>
     <row r="8" ht="26" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
@@ -800,6 +859,8 @@
           <t>Saturday, August 15, 2026 (final check-in — defense-ready)</t>
         </is>
       </c>
+      <c r="C8" s="46" t="n"/>
+      <c r="D8" s="47" t="n"/>
     </row>
     <row r="9" ht="26" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
@@ -812,6 +873,8 @@
           <t>Strict. Deadlines are gates — a task is not done until QA (Dave) signs off.</t>
         </is>
       </c>
+      <c r="C9" s="46" t="n"/>
+      <c r="D9" s="47" t="n"/>
     </row>
     <row r="10" ht="26" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
@@ -824,6 +887,8 @@
           <t>github.com/andrei13spot/smartcommuteph</t>
         </is>
       </c>
+      <c r="C10" s="46" t="n"/>
+      <c r="D10" s="47" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
@@ -831,6 +896,9 @@
           <t>Owners</t>
         </is>
       </c>
+      <c r="B12" s="46" t="n"/>
+      <c r="C12" s="46" t="n"/>
+      <c r="D12" s="47" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
@@ -940,6 +1008,9 @@
           <t>Status legend</t>
         </is>
       </c>
+      <c r="B19" s="46" t="n"/>
+      <c r="C19" s="46" t="n"/>
+      <c r="D19" s="47" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="12" t="inlineStr">
@@ -1028,6 +1099,8 @@
           <t>Before you start ANY task — always:</t>
         </is>
       </c>
+      <c r="B4" s="46" t="n"/>
+      <c r="C4" s="47" t="n"/>
     </row>
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="18" t="inlineStr">
@@ -1035,6 +1108,8 @@
           <t>git checkout dev</t>
         </is>
       </c>
+      <c r="B5" s="46" t="n"/>
+      <c r="C5" s="47" t="n"/>
     </row>
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="18" t="inlineStr">
@@ -1042,6 +1117,8 @@
           <t>git pull origin dev</t>
         </is>
       </c>
+      <c r="B6" s="46" t="n"/>
+      <c r="C6" s="47" t="n"/>
     </row>
     <row r="7" ht="20" customHeight="1">
       <c r="A7" s="18" t="inlineStr">
@@ -1049,6 +1126,8 @@
           <t>git checkout -b &lt;branch&gt;   # branch off the latest dev</t>
         </is>
       </c>
+      <c r="B7" s="46" t="n"/>
+      <c r="C7" s="47" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
@@ -1209,6 +1288,8 @@
           <t>• Commit small and often; lowercase messages.</t>
         </is>
       </c>
+      <c r="B20" s="46" t="n"/>
+      <c r="C20" s="47" t="n"/>
     </row>
     <row r="21" ht="22" customHeight="1">
       <c r="A21" s="22" t="inlineStr">
@@ -1216,6 +1297,8 @@
           <t>• Push your branch: git push -u origin &lt;branch&gt;.</t>
         </is>
       </c>
+      <c r="B21" s="46" t="n"/>
+      <c r="C21" s="47" t="n"/>
     </row>
     <row r="22" ht="22" customHeight="1">
       <c r="A22" s="22" t="inlineStr">
@@ -1223,6 +1306,8 @@
           <t>• Open a Pull Request into dev. Dave (QA) reviews &amp; signs off BEFORE it merges into dev.</t>
         </is>
       </c>
+      <c r="B22" s="46" t="n"/>
+      <c r="C22" s="47" t="n"/>
     </row>
     <row r="23" ht="22" customHeight="1">
       <c r="A23" s="22" t="inlineStr">
@@ -1230,6 +1315,8 @@
           <t>• Release: dev -&gt; main only at the Saturday check-in gates, once QA has signed off.</t>
         </is>
       </c>
+      <c r="B23" s="46" t="n"/>
+      <c r="C23" s="47" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -1238,8 +1325,8 @@
     <mergeCell ref="A23:C23"/>
     <mergeCell ref="A6:C6"/>
     <mergeCell ref="A22:C22"/>
+    <mergeCell ref="A21:C21"/>
     <mergeCell ref="A7:C7"/>
-    <mergeCell ref="A21:C21"/>
     <mergeCell ref="A4:C4"/>
     <mergeCell ref="A20:C20"/>
     <mergeCell ref="A2:C2"/>
@@ -1539,10 +1626,10 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="F5" s="28" t="n">
+      <c r="F5" s="48" t="n">
         <v>46216</v>
       </c>
-      <c r="G5" s="28" t="n">
+      <c r="G5" s="48" t="n">
         <v>46216</v>
       </c>
       <c r="H5" s="8" t="inlineStr">
@@ -1575,10 +1662,10 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="F6" s="28" t="n">
+      <c r="F6" s="48" t="n">
         <v>46216</v>
       </c>
-      <c r="G6" s="28" t="n">
+      <c r="G6" s="48" t="n">
         <v>46218</v>
       </c>
       <c r="H6" s="8" t="inlineStr">
@@ -1611,10 +1698,10 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="F7" s="28" t="n">
+      <c r="F7" s="48" t="n">
         <v>46217</v>
       </c>
-      <c r="G7" s="28" t="n">
+      <c r="G7" s="48" t="n">
         <v>46218</v>
       </c>
       <c r="H7" s="8" t="inlineStr">
@@ -1647,10 +1734,10 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="F8" s="28" t="n">
+      <c r="F8" s="48" t="n">
         <v>46218</v>
       </c>
-      <c r="G8" s="28" t="n">
+      <c r="G8" s="48" t="n">
         <v>46219</v>
       </c>
       <c r="H8" s="8" t="inlineStr">
@@ -1683,10 +1770,10 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="F9" s="28" t="n">
+      <c r="F9" s="48" t="n">
         <v>46219</v>
       </c>
-      <c r="G9" s="28" t="n">
+      <c r="G9" s="48" t="n">
         <v>46220</v>
       </c>
       <c r="H9" s="8" t="inlineStr">
@@ -1719,10 +1806,10 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="F10" s="28" t="n">
+      <c r="F10" s="48" t="n">
         <v>46220</v>
       </c>
-      <c r="G10" s="28" t="n">
+      <c r="G10" s="48" t="n">
         <v>46221</v>
       </c>
       <c r="H10" s="8" t="inlineStr">
@@ -1755,10 +1842,10 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="F11" s="28" t="n">
+      <c r="F11" s="48" t="n">
         <v>46220</v>
       </c>
-      <c r="G11" s="28" t="n">
+      <c r="G11" s="48" t="n">
         <v>46221</v>
       </c>
       <c r="H11" s="8" t="inlineStr">
@@ -1791,10 +1878,10 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="F12" s="28" t="n">
+      <c r="F12" s="48" t="n">
         <v>46218</v>
       </c>
-      <c r="G12" s="28" t="n">
+      <c r="G12" s="48" t="n">
         <v>46221</v>
       </c>
       <c r="H12" s="8" t="inlineStr">
@@ -1809,7 +1896,7 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Copy fixes: drop 'reimagined' &amp; 'live PAGASA' -&gt; 'PAGASA TenDay Forecast', framework voice</t>
+          <t>Copy fixes: drop 'reimagined' &amp; the 'live weather' wording -&gt; 'MET Norway rainfall forecast', framework voice</t>
         </is>
       </c>
       <c r="C13" s="29" t="inlineStr">
@@ -1827,10 +1914,10 @@
           <t>P2</t>
         </is>
       </c>
-      <c r="F13" s="28" t="n">
+      <c r="F13" s="48" t="n">
         <v>46221</v>
       </c>
-      <c r="G13" s="28" t="n">
+      <c r="G13" s="48" t="n">
         <v>46221</v>
       </c>
       <c r="H13" s="8" t="inlineStr">
@@ -1863,10 +1950,10 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="F14" s="35" t="n">
+      <c r="F14" s="49" t="n">
         <v>46221</v>
       </c>
-      <c r="G14" s="35" t="n">
+      <c r="G14" s="49" t="n">
         <v>46221</v>
       </c>
       <c r="H14" s="31" t="inlineStr">
@@ -1899,10 +1986,10 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="F15" s="28" t="n">
+      <c r="F15" s="48" t="n">
         <v>46223</v>
       </c>
-      <c r="G15" s="28" t="n">
+      <c r="G15" s="48" t="n">
         <v>46228</v>
       </c>
       <c r="H15" s="8" t="inlineStr">
@@ -1935,10 +2022,10 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="F16" s="28" t="n">
+      <c r="F16" s="48" t="n">
         <v>46230</v>
       </c>
-      <c r="G16" s="28" t="n">
+      <c r="G16" s="48" t="n">
         <v>46235</v>
       </c>
       <c r="H16" s="8" t="inlineStr">
@@ -1971,10 +2058,10 @@
           <t>P2</t>
         </is>
       </c>
-      <c r="F17" s="28" t="n">
+      <c r="F17" s="48" t="n">
         <v>46237</v>
       </c>
-      <c r="G17" s="28" t="n">
+      <c r="G17" s="48" t="n">
         <v>46242</v>
       </c>
       <c r="H17" s="8" t="inlineStr">
@@ -2007,10 +2094,10 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="F18" s="28" t="n">
+      <c r="F18" s="48" t="n">
         <v>46216</v>
       </c>
-      <c r="G18" s="28" t="n">
+      <c r="G18" s="48" t="n">
         <v>46218</v>
       </c>
       <c r="H18" s="8" t="inlineStr">
@@ -2043,10 +2130,10 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="F19" s="28" t="n">
+      <c r="F19" s="48" t="n">
         <v>46218</v>
       </c>
-      <c r="G19" s="28" t="n">
+      <c r="G19" s="48" t="n">
         <v>46220</v>
       </c>
       <c r="H19" s="8" t="inlineStr">
@@ -2079,10 +2166,10 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="F20" s="28" t="n">
+      <c r="F20" s="48" t="n">
         <v>46219</v>
       </c>
-      <c r="G20" s="28" t="n">
+      <c r="G20" s="48" t="n">
         <v>46221</v>
       </c>
       <c r="H20" s="8" t="inlineStr">
@@ -2115,10 +2202,10 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="F21" s="28" t="n">
+      <c r="F21" s="48" t="n">
         <v>46223</v>
       </c>
-      <c r="G21" s="28" t="n">
+      <c r="G21" s="48" t="n">
         <v>46225</v>
       </c>
       <c r="H21" s="8" t="inlineStr">
@@ -2151,10 +2238,10 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="F22" s="28" t="n">
+      <c r="F22" s="48" t="n">
         <v>46225</v>
       </c>
-      <c r="G22" s="28" t="n">
+      <c r="G22" s="48" t="n">
         <v>46226</v>
       </c>
       <c r="H22" s="8" t="inlineStr">
@@ -2187,10 +2274,10 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="F23" s="28" t="n">
+      <c r="F23" s="48" t="n">
         <v>46226</v>
       </c>
-      <c r="G23" s="28" t="n">
+      <c r="G23" s="48" t="n">
         <v>46227</v>
       </c>
       <c r="H23" s="8" t="inlineStr">
@@ -2223,10 +2310,10 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="F24" s="28" t="n">
+      <c r="F24" s="48" t="n">
         <v>46226</v>
       </c>
-      <c r="G24" s="28" t="n">
+      <c r="G24" s="48" t="n">
         <v>46227</v>
       </c>
       <c r="H24" s="8" t="inlineStr">
@@ -2259,10 +2346,10 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="F25" s="28" t="n">
+      <c r="F25" s="48" t="n">
         <v>46227</v>
       </c>
-      <c r="G25" s="28" t="n">
+      <c r="G25" s="48" t="n">
         <v>46228</v>
       </c>
       <c r="H25" s="8" t="inlineStr">
@@ -2295,10 +2382,10 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="F26" s="28" t="n">
+      <c r="F26" s="48" t="n">
         <v>46227</v>
       </c>
-      <c r="G26" s="28" t="n">
+      <c r="G26" s="48" t="n">
         <v>46228</v>
       </c>
       <c r="H26" s="8" t="inlineStr">
@@ -2331,10 +2418,10 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="F27" s="28" t="n">
+      <c r="F27" s="48" t="n">
         <v>46223</v>
       </c>
-      <c r="G27" s="28" t="n">
+      <c r="G27" s="48" t="n">
         <v>46232</v>
       </c>
       <c r="H27" s="8" t="inlineStr">
@@ -2349,7 +2436,7 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>RFR flood-risk model (scikit-learn, PAGASA TenDay Forecast input)</t>
+          <t>RFR flood-risk model (scikit-learn, MET Norway Locationforecast 24-hour rainfall input)</t>
         </is>
       </c>
       <c r="C28" s="36" t="inlineStr">
@@ -2367,10 +2454,10 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="F28" s="28" t="n">
+      <c r="F28" s="48" t="n">
         <v>46225</v>
       </c>
-      <c r="G28" s="28" t="n">
+      <c r="G28" s="48" t="n">
         <v>46232</v>
       </c>
       <c r="H28" s="8" t="inlineStr">
@@ -2403,10 +2490,10 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="F29" s="28" t="n">
+      <c r="F29" s="48" t="n">
         <v>46232</v>
       </c>
-      <c r="G29" s="28" t="n">
+      <c r="G29" s="48" t="n">
         <v>46233</v>
       </c>
       <c r="H29" s="8" t="inlineStr">
@@ -2439,10 +2526,10 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="F30" s="28" t="n">
+      <c r="F30" s="48" t="n">
         <v>46233</v>
       </c>
-      <c r="G30" s="28" t="n">
+      <c r="G30" s="48" t="n">
         <v>46235</v>
       </c>
       <c r="H30" s="8" t="inlineStr">
@@ -2475,10 +2562,10 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="F31" s="28" t="n">
+      <c r="F31" s="48" t="n">
         <v>46237</v>
       </c>
-      <c r="G31" s="28" t="n">
+      <c r="G31" s="48" t="n">
         <v>46242</v>
       </c>
       <c r="H31" s="8" t="inlineStr">
@@ -2511,10 +2598,10 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="F32" s="28" t="n">
+      <c r="F32" s="48" t="n">
         <v>46216</v>
       </c>
-      <c r="G32" s="28" t="n">
+      <c r="G32" s="48" t="n">
         <v>46223</v>
       </c>
       <c r="H32" s="8" t="inlineStr">
@@ -2547,10 +2634,10 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="F33" s="28" t="n">
+      <c r="F33" s="48" t="n">
         <v>46223</v>
       </c>
-      <c r="G33" s="28" t="n">
+      <c r="G33" s="48" t="n">
         <v>46223</v>
       </c>
       <c r="H33" s="8" t="inlineStr">
@@ -2583,10 +2670,10 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="F34" s="28" t="n">
+      <c r="F34" s="48" t="n">
         <v>46219</v>
       </c>
-      <c r="G34" s="28" t="n">
+      <c r="G34" s="48" t="n">
         <v>46221</v>
       </c>
       <c r="H34" s="8" t="inlineStr">
@@ -2619,10 +2706,10 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="F35" s="28" t="n">
+      <c r="F35" s="48" t="n">
         <v>46218</v>
       </c>
-      <c r="G35" s="28" t="n">
+      <c r="G35" s="48" t="n">
         <v>46223</v>
       </c>
       <c r="H35" s="8" t="inlineStr">
@@ -2655,10 +2742,10 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="F36" s="28" t="n">
+      <c r="F36" s="48" t="n">
         <v>46225</v>
       </c>
-      <c r="G36" s="28" t="n">
+      <c r="G36" s="48" t="n">
         <v>46232</v>
       </c>
       <c r="H36" s="8" t="inlineStr">
@@ -2691,10 +2778,10 @@
           <t>P2</t>
         </is>
       </c>
-      <c r="F37" s="28" t="n">
+      <c r="F37" s="48" t="n">
         <v>46230</v>
       </c>
-      <c r="G37" s="28" t="n">
+      <c r="G37" s="48" t="n">
         <v>46242</v>
       </c>
       <c r="H37" s="8" t="inlineStr">
@@ -2727,10 +2814,10 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="F38" s="28" t="n">
+      <c r="F38" s="48" t="n">
         <v>46218</v>
       </c>
-      <c r="G38" s="28" t="n">
+      <c r="G38" s="48" t="n">
         <v>46221</v>
       </c>
       <c r="H38" s="8" t="inlineStr">
@@ -2763,10 +2850,10 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="F39" s="28" t="n">
+      <c r="F39" s="48" t="n">
         <v>46221</v>
       </c>
-      <c r="G39" s="28" t="n">
+      <c r="G39" s="48" t="n">
         <v>46223</v>
       </c>
       <c r="H39" s="8" t="inlineStr">
@@ -2799,10 +2886,10 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="F40" s="28" t="n">
+      <c r="F40" s="48" t="n">
         <v>46223</v>
       </c>
-      <c r="G40" s="28" t="n">
+      <c r="G40" s="48" t="n">
         <v>46228</v>
       </c>
       <c r="H40" s="8" t="inlineStr">
@@ -2835,10 +2922,10 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="F41" s="28" t="n">
+      <c r="F41" s="48" t="n">
         <v>46230</v>
       </c>
-      <c r="G41" s="28" t="n">
+      <c r="G41" s="48" t="n">
         <v>46234</v>
       </c>
       <c r="H41" s="8" t="inlineStr">
@@ -2871,10 +2958,10 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="F42" s="28" t="n">
+      <c r="F42" s="48" t="n">
         <v>46234</v>
       </c>
-      <c r="G42" s="28" t="n">
+      <c r="G42" s="48" t="n">
         <v>46235</v>
       </c>
       <c r="H42" s="8" t="inlineStr">
@@ -2907,10 +2994,10 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="F43" s="28" t="n">
+      <c r="F43" s="48" t="n">
         <v>46237</v>
       </c>
-      <c r="G43" s="28" t="n">
+      <c r="G43" s="48" t="n">
         <v>46238</v>
       </c>
       <c r="H43" s="8" t="inlineStr">
@@ -2943,10 +3030,10 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="F44" s="28" t="n">
+      <c r="F44" s="48" t="n">
         <v>46238</v>
       </c>
-      <c r="G44" s="28" t="n">
+      <c r="G44" s="48" t="n">
         <v>46239</v>
       </c>
       <c r="H44" s="8" t="inlineStr">
@@ -2979,10 +3066,10 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="F45" s="28" t="n">
+      <c r="F45" s="48" t="n">
         <v>46240</v>
       </c>
-      <c r="G45" s="28" t="n">
+      <c r="G45" s="48" t="n">
         <v>46242</v>
       </c>
       <c r="H45" s="8" t="inlineStr">
@@ -3015,10 +3102,10 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="F46" s="28" t="n">
+      <c r="F46" s="48" t="n">
         <v>46242</v>
       </c>
-      <c r="G46" s="28" t="n">
+      <c r="G46" s="48" t="n">
         <v>46242</v>
       </c>
       <c r="H46" s="8" t="inlineStr">
@@ -3051,10 +3138,10 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="F47" s="28" t="n">
+      <c r="F47" s="48" t="n">
         <v>46244</v>
       </c>
-      <c r="G47" s="28" t="n">
+      <c r="G47" s="48" t="n">
         <v>46249</v>
       </c>
       <c r="H47" s="8" t="inlineStr">
@@ -3087,10 +3174,10 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="F48" s="35" t="n">
+      <c r="F48" s="49" t="n">
         <v>46249</v>
       </c>
-      <c r="G48" s="35" t="n">
+      <c r="G48" s="49" t="n">
         <v>46249</v>
       </c>
       <c r="H48" s="31" t="inlineStr">
@@ -3305,6 +3392,7 @@
           <t>POST /route</t>
         </is>
       </c>
+      <c r="B5" s="47" t="n"/>
     </row>
     <row r="6" ht="40" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
@@ -3360,6 +3448,7 @@
           <t>POST /compare</t>
         </is>
       </c>
+      <c r="B10" s="47" t="n"/>
     </row>
     <row r="11" ht="40" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
@@ -3403,6 +3492,7 @@
           <t>Benchmark log</t>
         </is>
       </c>
+      <c r="B14" s="47" t="n"/>
     </row>
     <row r="15" ht="40" customHeight="1">
       <c r="A15" s="3" t="inlineStr">

</xml_diff>